<commit_message>
June Temp and Room Temp Success
</commit_message>
<xml_diff>
--- a/Data/Excel/Measurement.xlsx
+++ b/Data/Excel/Measurement.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Senior Project\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Senior Project\Data\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6EC7208B-1B15-47FA-B4B1-68CAD2020112}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50A63F94-1019-41FE-A2AC-396454CC09EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1560" yWindow="1560" windowWidth="21600" windowHeight="11295" firstSheet="2" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="2" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hourly Room Temp" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="484" uniqueCount="436">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="483" uniqueCount="435">
   <si>
     <t>position</t>
   </si>
@@ -1346,10 +1346,7 @@
     <t>T2</t>
   </si>
   <si>
-    <t>Temp1</t>
-  </si>
-  <si>
-    <t>Temp2</t>
+    <t>Temp_Room_Air</t>
   </si>
 </sst>
 </file>
@@ -24461,799 +24458,583 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BE050A31-C028-4E8C-AE92-C9A8CD5F1DD2}">
-  <dimension ref="A1:C72"/>
+  <dimension ref="A1:B72"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>427</v>
       </c>
       <c r="B1" t="s">
         <v>434</v>
       </c>
-      <c r="C1" t="s">
-        <v>435</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>0</v>
       </c>
       <c r="B2">
-        <v>27.1</v>
-      </c>
-      <c r="C2">
-        <v>27.1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+        <v>28.7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>60</v>
       </c>
       <c r="B3">
-        <v>26.9</v>
-      </c>
-      <c r="C3">
-        <v>26.7</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+        <v>28.6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>120</v>
       </c>
       <c r="B4">
-        <v>26.7</v>
-      </c>
-      <c r="C4">
-        <v>26.3</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+        <v>28.6</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>180</v>
       </c>
       <c r="B5">
-        <v>26.5</v>
-      </c>
-      <c r="C5">
-        <v>25.8</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+        <v>28.5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>240</v>
       </c>
       <c r="B6">
-        <v>26.2</v>
-      </c>
-      <c r="C6">
-        <v>25.5</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+        <v>28.4</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>300</v>
       </c>
       <c r="B7">
-        <v>25.7</v>
-      </c>
-      <c r="C7">
-        <v>25.1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+        <v>28.2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>360</v>
       </c>
       <c r="B8">
-        <v>25.2</v>
-      </c>
-      <c r="C8">
-        <v>24.7</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+        <v>27.9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>420</v>
       </c>
       <c r="B9">
-        <v>24.8</v>
-      </c>
-      <c r="C9">
-        <v>24.3</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+        <v>27.5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>480</v>
       </c>
       <c r="B10">
-        <v>24.3</v>
-      </c>
-      <c r="C10">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
+        <v>27.1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>540</v>
       </c>
       <c r="B11">
-        <v>23.9</v>
-      </c>
-      <c r="C11">
-        <v>23.7</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
+        <v>26.7</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>600</v>
       </c>
       <c r="B12">
-        <v>23.3</v>
-      </c>
-      <c r="C12">
-        <v>23.4</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
+        <v>26.3</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>660</v>
       </c>
       <c r="B13">
-        <v>23.2</v>
-      </c>
-      <c r="C13">
-        <v>23.1</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
+        <v>25.8</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>720</v>
       </c>
       <c r="B14">
-        <v>22.8</v>
-      </c>
-      <c r="C14">
-        <v>22.8</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
+        <v>25.5</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>780</v>
       </c>
       <c r="B15">
-        <v>22.4</v>
-      </c>
-      <c r="C15">
-        <v>22.7</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
+        <v>25.1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>840</v>
       </c>
       <c r="B16">
-        <v>22.1</v>
-      </c>
-      <c r="C16">
-        <v>22.5</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
+        <v>24.7</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A17">
         <v>900</v>
       </c>
       <c r="B17">
-        <v>21.8</v>
-      </c>
-      <c r="C17">
-        <v>22.3</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
+        <v>24.3</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A18">
         <v>960</v>
       </c>
       <c r="B18">
-        <v>21.5</v>
-      </c>
-      <c r="C18">
-        <v>22.1</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A19">
         <v>1020</v>
       </c>
       <c r="B19">
-        <v>21.3</v>
-      </c>
-      <c r="C19">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
+        <v>23.7</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A20">
         <v>1080</v>
       </c>
       <c r="B20">
-        <v>21.1</v>
-      </c>
-      <c r="C20">
-        <v>21.9</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
+        <v>23.4</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A21">
         <v>1140</v>
       </c>
       <c r="B21">
-        <v>21.1</v>
-      </c>
-      <c r="C21">
-        <v>21.8</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
+        <v>23.1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A22">
         <v>1200</v>
       </c>
       <c r="B22">
-        <v>21.2</v>
-      </c>
-      <c r="C22">
-        <v>21.8</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
+        <v>22.8</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A23">
         <v>1260</v>
       </c>
       <c r="B23">
-        <v>21.3</v>
-      </c>
-      <c r="C23">
-        <v>21.8</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
+        <v>22.7</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A24">
         <v>1320</v>
       </c>
       <c r="B24">
-        <v>21.4</v>
-      </c>
-      <c r="C24">
-        <v>21.8</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
+        <v>22.5</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A25">
         <v>1380</v>
       </c>
       <c r="B25">
-        <v>21.5</v>
-      </c>
-      <c r="C25">
-        <v>21.7</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
+        <v>22.3</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A26">
         <v>1440</v>
       </c>
       <c r="B26">
-        <v>21.6</v>
-      </c>
-      <c r="C26">
-        <v>21.6</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.2">
+        <v>22.1</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A27">
         <v>1500</v>
       </c>
       <c r="B27">
-        <v>21.6</v>
-      </c>
-      <c r="C27">
-        <v>21.5</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.2">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A28">
         <v>1560</v>
       </c>
       <c r="B28">
-        <v>21.5</v>
-      </c>
-      <c r="C28">
-        <v>21.4</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.2">
+        <v>21.9</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A29">
         <v>1620</v>
       </c>
       <c r="B29">
-        <v>21.5</v>
-      </c>
-      <c r="C29">
-        <v>21.2</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.2">
+        <v>21.8</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A30">
         <v>1680</v>
       </c>
       <c r="B30">
-        <v>21.6</v>
-      </c>
-      <c r="C30">
-        <v>21.2</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.2">
+        <v>21.8</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A31">
         <v>1740</v>
       </c>
       <c r="B31">
-        <v>21.7</v>
-      </c>
-      <c r="C31">
-        <v>21.2</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.2">
+        <v>21.8</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A32">
         <v>1800</v>
       </c>
       <c r="B32">
         <v>21.8</v>
       </c>
-      <c r="C32">
-        <v>21.2</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.2">
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A33">
         <v>1860</v>
       </c>
       <c r="B33">
-        <v>21.9</v>
-      </c>
-      <c r="C33">
-        <v>21.2</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.2">
+        <v>21.7</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A34">
         <v>1920</v>
       </c>
       <c r="B34">
-        <v>21.9</v>
-      </c>
-      <c r="C34">
-        <v>21.2</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.2">
+        <v>21.6</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A35">
         <v>1980</v>
       </c>
       <c r="B35">
-        <v>22</v>
-      </c>
-      <c r="C35">
-        <v>21.2</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.2">
+        <v>21.5</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A36">
         <v>2040</v>
       </c>
       <c r="B36">
-        <v>22</v>
-      </c>
-      <c r="C36">
-        <v>21.1</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.2">
+        <v>21.4</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A37">
         <v>2100</v>
       </c>
       <c r="B37">
-        <v>22.1</v>
-      </c>
-      <c r="C37">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.2">
+        <v>21.2</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A38">
         <v>2160</v>
       </c>
       <c r="B38">
-        <v>22.1</v>
-      </c>
-      <c r="C38">
-        <v>20.9</v>
-      </c>
-    </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.2">
+        <v>21.2</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A39">
         <v>2220</v>
       </c>
       <c r="B39">
-        <v>22.1</v>
-      </c>
-      <c r="C39">
-        <v>20.9</v>
-      </c>
-    </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.2">
+        <v>21.2</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A40">
         <v>2280</v>
       </c>
       <c r="B40">
-        <v>22</v>
-      </c>
-      <c r="C40">
-        <v>20.9</v>
-      </c>
-    </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.2">
+        <v>21.2</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A41">
         <v>2340</v>
       </c>
       <c r="B41">
-        <v>22</v>
-      </c>
-      <c r="C41">
-        <v>20.9</v>
-      </c>
-    </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.2">
+        <v>21.2</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A42">
         <v>2400</v>
       </c>
       <c r="B42">
-        <v>21.9</v>
-      </c>
-      <c r="C42">
-        <v>20.9</v>
-      </c>
-    </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.2">
+        <v>21.2</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A43">
         <v>2460</v>
       </c>
       <c r="B43">
-        <v>21.9</v>
-      </c>
-      <c r="C43">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.2">
+        <v>21.2</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A44">
         <v>2520</v>
       </c>
       <c r="B44">
-        <v>21.9</v>
-      </c>
-      <c r="C44">
         <v>21.1</v>
       </c>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A45">
         <v>2580</v>
       </c>
       <c r="B45">
-        <v>21.8</v>
-      </c>
-      <c r="C45">
         <v>21</v>
       </c>
     </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A46">
         <v>2640</v>
       </c>
       <c r="B46">
-        <v>21.6</v>
-      </c>
-      <c r="C46">
         <v>20.9</v>
       </c>
     </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A47">
         <v>2700</v>
       </c>
       <c r="B47">
-        <v>21.5</v>
-      </c>
-      <c r="C47">
-        <v>20.7</v>
-      </c>
-    </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.2">
+        <v>20.9</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A48">
         <v>2760</v>
       </c>
       <c r="B48">
-        <v>21.5</v>
-      </c>
-      <c r="C48">
-        <v>20.7</v>
-      </c>
-    </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.2">
+        <v>20.9</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A49">
         <v>2820</v>
       </c>
       <c r="B49">
-        <v>21.4</v>
-      </c>
-      <c r="C49">
-        <v>20.7</v>
-      </c>
-    </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.2">
+        <v>20.9</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A50">
         <v>2880</v>
       </c>
       <c r="B50">
-        <v>21.5</v>
-      </c>
-      <c r="C50">
-        <v>20.8</v>
-      </c>
-    </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.2">
+        <v>20.9</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A51">
         <v>2940</v>
       </c>
       <c r="B51">
-        <v>21.5</v>
-      </c>
-      <c r="C51">
-        <v>20.8</v>
-      </c>
-    </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.2">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A52">
         <v>3000</v>
       </c>
       <c r="B52">
-        <v>21.5</v>
-      </c>
-      <c r="C52">
-        <v>20.8</v>
-      </c>
-    </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.2">
+        <v>21.1</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A53">
         <v>3060</v>
       </c>
       <c r="B53">
-        <v>21.6</v>
-      </c>
-      <c r="C53">
-        <v>20.8</v>
-      </c>
-    </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.2">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A54">
         <v>3120</v>
       </c>
       <c r="B54">
-        <v>21.6</v>
-      </c>
-      <c r="C54">
-        <v>20.8</v>
-      </c>
-    </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.2">
+        <v>20.9</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A55">
         <v>3180</v>
       </c>
       <c r="B55">
-        <v>21.6</v>
-      </c>
-      <c r="C55">
         <v>20.7</v>
       </c>
     </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A56">
         <v>3240</v>
       </c>
       <c r="B56">
-        <v>21.7</v>
-      </c>
-      <c r="C56">
-        <v>20.5</v>
-      </c>
-    </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.2">
+        <v>20.7</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A57">
         <v>3300</v>
       </c>
       <c r="B57">
-        <v>21.6</v>
-      </c>
-      <c r="C57">
-        <v>20.5</v>
-      </c>
-    </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.2">
+        <v>20.7</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A58">
         <v>3360</v>
       </c>
       <c r="B58">
-        <v>21.6</v>
-      </c>
-      <c r="C58">
-        <v>20.6</v>
-      </c>
-    </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.2">
+        <v>20.8</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A59">
         <v>3420</v>
       </c>
       <c r="B59">
-        <v>21.5</v>
-      </c>
-      <c r="C59">
-        <v>20.7</v>
-      </c>
-    </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.2">
+        <v>20.8</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A60">
         <v>3480</v>
       </c>
       <c r="B60">
-        <v>21.6</v>
-      </c>
-      <c r="C60">
         <v>20.8</v>
       </c>
     </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A61">
         <v>3540</v>
       </c>
       <c r="B61">
-        <v>21.6</v>
-      </c>
-      <c r="C61">
         <v>20.8</v>
       </c>
     </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A62">
         <v>3600</v>
       </c>
       <c r="B62">
-        <v>21.6</v>
-      </c>
-      <c r="C62">
         <v>20.8</v>
       </c>
     </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A63">
         <v>3660</v>
       </c>
       <c r="B63">
-        <v>21.6</v>
-      </c>
-      <c r="C63">
-        <v>20.9</v>
-      </c>
-    </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.2">
+        <v>20.7</v>
+      </c>
+    </row>
+    <row r="64" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A64">
         <v>3720</v>
       </c>
       <c r="B64">
-        <v>21.6</v>
-      </c>
-      <c r="C64">
-        <v>20.9</v>
-      </c>
-    </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.2">
+        <v>20.5</v>
+      </c>
+    </row>
+    <row r="65" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A65">
         <v>3780</v>
       </c>
       <c r="B65">
-        <v>21.5</v>
-      </c>
-      <c r="C65">
         <v>20.5</v>
       </c>
     </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A66">
         <v>3840</v>
       </c>
       <c r="B66">
-        <v>21.5</v>
-      </c>
-      <c r="C66">
         <v>20.6</v>
       </c>
     </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A67">
         <v>3900</v>
       </c>
       <c r="B67">
-        <v>21.5</v>
-      </c>
-      <c r="C67">
         <v>20.7</v>
       </c>
     </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A68">
         <v>3960</v>
       </c>
       <c r="B68">
-        <v>21.5</v>
-      </c>
-      <c r="C68">
-        <v>20.8</v>
-      </c>
-    </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.2">
+        <v>20.7</v>
+      </c>
+    </row>
+    <row r="69" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A69">
         <v>4020</v>
       </c>
       <c r="B69">
-        <v>21.6</v>
-      </c>
-      <c r="C69">
-        <v>20.8</v>
-      </c>
-    </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.2">
+        <v>20.7</v>
+      </c>
+    </row>
+    <row r="70" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A70">
         <v>4080</v>
       </c>
       <c r="B70">
-        <v>21.6</v>
-      </c>
-      <c r="C70">
-        <v>20.8</v>
-      </c>
-    </row>
-    <row r="71" spans="1:3" x14ac:dyDescent="0.2">
+        <v>20.7</v>
+      </c>
+    </row>
+    <row r="71" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A71">
         <v>4140</v>
       </c>
       <c r="B71">
-        <v>21.5</v>
-      </c>
-      <c r="C71">
-        <v>20.9</v>
-      </c>
-    </row>
-    <row r="72" spans="1:3" x14ac:dyDescent="0.2">
+        <v>20.7</v>
+      </c>
+    </row>
+    <row r="72" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A72">
         <v>4200</v>
       </c>
       <c r="B72">
-        <v>21.5</v>
-      </c>
-      <c r="C72">
-        <v>20.9</v>
+        <v>20.7</v>
       </c>
     </row>
   </sheetData>
@@ -25424,26 +25205,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="228fa7ca-c38f-4560-861c-8ff0895b344f">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="60441c17-193d-4aaa-84fe-076df351db0c" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101004A83FCAD2B02494AB70746B544CC61AE" ma:contentTypeVersion="10" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="77bfa71e1908209a377d80d9948cd243">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="228fa7ca-c38f-4560-861c-8ff0895b344f" xmlns:ns3="60441c17-193d-4aaa-84fe-076df351db0c" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="cf08252bb5eb797fcd948f11b977b465" ns2:_="" ns3:_="">
     <xsd:import namespace="228fa7ca-c38f-4560-861c-8ff0895b344f"/>
@@ -25632,26 +25393,27 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DBA7AD0B-D9B0-45DE-A7AE-8A303D13225D}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="228fa7ca-c38f-4560-861c-8ff0895b344f"/>
-    <ds:schemaRef ds:uri="60441c17-193d-4aaa-84fe-076df351db0c"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{94823659-B512-4ECA-9D86-4915201F8F7B}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="228fa7ca-c38f-4560-861c-8ff0895b344f">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="60441c17-193d-4aaa-84fe-076df351db0c" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D94FF3E2-982E-40E4-B192-D71C6EF31E2D}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -25668,4 +25430,23 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{94823659-B512-4ECA-9D86-4915201F8F7B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DBA7AD0B-D9B0-45DE-A7AE-8A303D13225D}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="228fa7ca-c38f-4560-861c-8ff0895b344f"/>
+    <ds:schemaRef ds:uri="60441c17-193d-4aaa-84fe-076df351db0c"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>